<commit_message>
Angle recorder change: virtual goniometer implemented for shoulder and elbow flexion
</commit_message>
<xml_diff>
--- a/Data_Analysis/IMU_Results.xlsx
+++ b/Data_Analysis/IMU_Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALUMNO\Desktop\CEU\4\Proyectos\IMU_Visualization\Data_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FC77D5-1D3B-4322-A8B5-C4A4D6636612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DD936B2-45FC-4C45-A7A5-46CF0E4D93E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subject_Metadata" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="49">
   <si>
     <t>Subject_ID</t>
   </si>
@@ -180,6 +180,15 @@
   </si>
   <si>
     <t>Male</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>muy preciso</t>
+  </si>
+  <si>
+    <t>with palm touches face, not fingers</t>
   </si>
 </sst>
 </file>
@@ -664,8 +673,12 @@
       <c r="D3" s="3">
         <v>195</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="E3" s="3">
+        <v>39.5</v>
+      </c>
+      <c r="F3" s="3">
+        <v>30</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
@@ -2454,8 +2467,12 @@
       <c r="B6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="C6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
@@ -2464,7 +2481,9 @@
       <c r="B7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="3"/>
+      <c r="C7" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -2474,7 +2493,9 @@
       <c r="B8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="3"/>
+      <c r="C8" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -2484,8 +2505,12 @@
       <c r="B9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="C9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">

</xml_diff>

<commit_message>
Data analysis ipynb changes
</commit_message>
<xml_diff>
--- a/Data_Analysis/IMU_Results.xlsx
+++ b/Data_Analysis/IMU_Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALUMNO\Desktop\CEU\4\Proyectos\IMU_Visualization\Data_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DD936B2-45FC-4C45-A7A5-46CF0E4D93E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB6A1CCB-E73D-4195-BBF4-51396C867B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subject_Metadata" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="63">
   <si>
     <t>Subject_ID</t>
   </si>
@@ -189,13 +189,78 @@
   </si>
   <si>
     <t>with palm touches face, not fingers</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>La lectura de ~159º en el rango máximo coincide con el límite anatómico real de la articulación glenohumeral, demostrando que el IMU aísla el movimiento del brazo sin sumar la compensación espinal del sujeto.</t>
+  </si>
+  <si>
+    <t>neutro</t>
+  </si>
+  <si>
+    <t>rot interna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rot externa </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Si pegas el codo a las costillas y rotas la mano hacia afuera (rotación externa) sin despegar el codo ni arquear la espalda, el rango articular medio en adultos sanos es de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>entre 45º y 60º</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Los 90º parte gira el omplato, el humero no gira 90</t>
+    </r>
+  </si>
+  <si>
+    <t>pronacion palma abajo</t>
+  </si>
+  <si>
+    <t>supinacion palma arriba</t>
+  </si>
+  <si>
+    <t>extension max hacia arriba</t>
+  </si>
+  <si>
+    <t>flexion max hacia abajo</t>
+  </si>
+  <si>
+    <t>desviacion a la izquierda, descordinacion radial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hiperflexion radiocubital </t>
+  </si>
+  <si>
+    <t>ligera desviacion radial izquierda</t>
+  </si>
+  <si>
+    <t>Macarena Querol</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -219,8 +284,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,6 +342,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -297,7 +388,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -307,6 +398,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -684,11 +778,21 @@
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="2">
+        <v>176</v>
+      </c>
+      <c r="E4" s="2">
+        <v>32</v>
+      </c>
+      <c r="F4" s="2">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:C4" xr:uid="{00000000-0009-0000-0000-000000000000}">
@@ -700,8 +804,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr codeName="Hoja2"/>
-  <dimension ref="A1:H64"/>
+  <sheetPr codeName="Hoja2" filterMode="1"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="16.7265625" customWidth="1"/>
@@ -730,7 +834,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
@@ -749,7 +853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
@@ -771,7 +875,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
@@ -790,7 +894,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
@@ -809,7 +913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -828,7 +932,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
@@ -847,7 +951,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>5</v>
       </c>
@@ -866,7 +970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>5</v>
       </c>
@@ -885,7 +989,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>5</v>
       </c>
@@ -904,7 +1008,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>5</v>
       </c>
@@ -923,7 +1027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>5</v>
       </c>
@@ -942,7 +1046,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>5</v>
       </c>
@@ -961,7 +1065,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>5</v>
       </c>
@@ -980,7 +1084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>5</v>
       </c>
@@ -999,7 +1103,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>5</v>
       </c>
@@ -1018,7 +1122,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
         <v>5</v>
       </c>
@@ -1037,7 +1141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
         <v>5</v>
       </c>
@@ -1056,7 +1160,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
         <v>5</v>
       </c>
@@ -1075,7 +1179,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
         <v>5</v>
       </c>
@@ -1094,7 +1198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>5</v>
       </c>
@@ -1113,7 +1217,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6" t="s">
         <v>5</v>
       </c>
@@ -1132,7 +1236,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>6</v>
       </c>
@@ -1145,13 +1249,15 @@
       <c r="D23" s="4">
         <v>0</v>
       </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E23" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F23" s="4" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>6</v>
       </c>
@@ -1164,13 +1270,16 @@
       <c r="D24" s="4">
         <v>90</v>
       </c>
-      <c r="E24" s="4"/>
+      <c r="E24" s="4">
+        <v>83.2</v>
+      </c>
       <c r="F24" s="4">
         <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+        <v>6.7999999999999972</v>
+      </c>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>6</v>
       </c>
@@ -1183,13 +1292,19 @@
       <c r="D25" s="4">
         <v>180</v>
       </c>
-      <c r="E25" s="4"/>
+      <c r="E25" s="4">
+        <v>158.80000000000001</v>
+      </c>
       <c r="F25" s="4">
         <f t="shared" si="0"/>
-        <v>180</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+        <v>21.199999999999989</v>
+      </c>
+      <c r="G25" s="11"/>
+      <c r="H25" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>6</v>
       </c>
@@ -1202,13 +1317,15 @@
       <c r="D26" s="4">
         <v>0</v>
       </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E26" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F26" s="4" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>6</v>
       </c>
@@ -1221,13 +1338,16 @@
       <c r="D27" s="4">
         <v>45</v>
       </c>
-      <c r="E27" s="4"/>
+      <c r="E27" s="4">
+        <v>49.6</v>
+      </c>
       <c r="F27" s="4">
         <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+        <v>4.6000000000000014</v>
+      </c>
+      <c r="G27" s="9"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>6</v>
       </c>
@@ -1240,13 +1360,16 @@
       <c r="D28" s="4">
         <v>90</v>
       </c>
-      <c r="E28" s="4"/>
+      <c r="E28" s="4">
+        <v>92.4</v>
+      </c>
       <c r="F28" s="4">
         <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+        <v>2.4000000000000057</v>
+      </c>
+      <c r="G28" s="9"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>6</v>
       </c>
@@ -1259,13 +1382,19 @@
       <c r="D29" s="4">
         <v>0</v>
       </c>
-      <c r="E29" s="4"/>
+      <c r="E29" s="4">
+        <v>44.7</v>
+      </c>
       <c r="F29" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+        <v>44.7</v>
+      </c>
+      <c r="G29" s="11"/>
+      <c r="H29" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>6</v>
       </c>
@@ -1278,13 +1407,22 @@
       <c r="D30" s="4">
         <v>90</v>
       </c>
-      <c r="E30" s="4"/>
+      <c r="E30" s="4">
+        <v>92.8</v>
+      </c>
       <c r="F30" s="4">
         <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+        <v>2.7999999999999972</v>
+      </c>
+      <c r="G30" s="9"/>
+      <c r="H30" t="s">
+        <v>51</v>
+      </c>
+      <c r="J30" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
         <v>6</v>
       </c>
@@ -1295,15 +1433,21 @@
         <v>18</v>
       </c>
       <c r="D31" s="4">
-        <v>-90</v>
-      </c>
-      <c r="E31" s="4"/>
+        <v>180</v>
+      </c>
+      <c r="E31" s="4">
+        <v>141.5</v>
+      </c>
       <c r="F31" s="4">
         <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+        <v>38.5</v>
+      </c>
+      <c r="G31" s="11"/>
+      <c r="H31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
         <v>6</v>
       </c>
@@ -1316,13 +1460,15 @@
       <c r="D32" s="5">
         <v>0</v>
       </c>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E32" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F32" s="5" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
         <v>6</v>
       </c>
@@ -1335,13 +1481,16 @@
       <c r="D33" s="5">
         <v>90</v>
       </c>
-      <c r="E33" s="5"/>
+      <c r="E33" s="5">
+        <v>66</v>
+      </c>
       <c r="F33" s="5">
         <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+      <c r="G33" s="11"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>6</v>
       </c>
@@ -1354,13 +1503,16 @@
       <c r="D34" s="5">
         <v>145</v>
       </c>
-      <c r="E34" s="5"/>
+      <c r="E34" s="5">
+        <v>117.7</v>
+      </c>
       <c r="F34" s="5">
         <f t="shared" si="0"/>
-        <v>145</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+        <v>27.299999999999997</v>
+      </c>
+      <c r="G34" s="11"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>6</v>
       </c>
@@ -1373,13 +1525,15 @@
       <c r="D35" s="5">
         <v>0</v>
       </c>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E35" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F35" s="5" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>6</v>
       </c>
@@ -1392,13 +1546,19 @@
       <c r="D36" s="5">
         <v>85</v>
       </c>
-      <c r="E36" s="5"/>
+      <c r="E36" s="5">
+        <v>67.2</v>
+      </c>
       <c r="F36" s="5">
         <f t="shared" si="0"/>
-        <v>85</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+        <v>17.799999999999997</v>
+      </c>
+      <c r="G36" s="11"/>
+      <c r="H36" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
         <v>6</v>
       </c>
@@ -1409,15 +1569,21 @@
         <v>19</v>
       </c>
       <c r="D37" s="5">
-        <v>-85</v>
-      </c>
-      <c r="E37" s="5"/>
+        <v>85</v>
+      </c>
+      <c r="E37" s="5">
+        <v>38.5</v>
+      </c>
       <c r="F37" s="5">
         <f t="shared" si="0"/>
-        <v>85</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+        <v>46.5</v>
+      </c>
+      <c r="G37" s="11"/>
+      <c r="H37" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
         <v>6</v>
       </c>
@@ -1436,7 +1602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
         <v>6</v>
       </c>
@@ -1449,13 +1615,19 @@
       <c r="D39" s="6">
         <v>70</v>
       </c>
-      <c r="E39" s="6"/>
+      <c r="E39" s="6">
+        <v>66.099999999999994</v>
+      </c>
       <c r="F39" s="6">
         <f t="shared" si="0"/>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+        <v>3.9000000000000057</v>
+      </c>
+      <c r="G39" s="9"/>
+      <c r="H39" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="6" t="s">
         <v>6</v>
       </c>
@@ -1466,15 +1638,21 @@
         <v>16</v>
       </c>
       <c r="D40" s="6">
-        <v>-70</v>
-      </c>
-      <c r="E40" s="6"/>
+        <v>70</v>
+      </c>
+      <c r="E40" s="6">
+        <v>53.2</v>
+      </c>
       <c r="F40" s="6">
         <f t="shared" si="0"/>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+        <v>16.799999999999997</v>
+      </c>
+      <c r="G40" s="11"/>
+      <c r="H40" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
         <v>6</v>
       </c>
@@ -1493,7 +1671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
         <v>6</v>
       </c>
@@ -1512,7 +1690,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
         <v>6</v>
       </c>
@@ -1531,7 +1709,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
         <v>7</v>
       </c>
@@ -1550,7 +1728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="s">
         <v>7</v>
       </c>
@@ -1569,7 +1747,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
         <v>7</v>
       </c>
@@ -1588,7 +1766,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
         <v>7</v>
       </c>
@@ -1607,7 +1785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
         <v>7</v>
       </c>
@@ -1626,7 +1804,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="4" t="s">
         <v>7</v>
       </c>
@@ -1645,7 +1823,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
         <v>7</v>
       </c>
@@ -1664,7 +1842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
         <v>7</v>
       </c>
@@ -1683,7 +1861,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="s">
         <v>7</v>
       </c>
@@ -1702,7 +1880,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>7</v>
       </c>
@@ -1721,7 +1899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
         <v>7</v>
       </c>
@@ -1740,7 +1918,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>7</v>
       </c>
@@ -1759,7 +1937,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>7</v>
       </c>
@@ -1778,7 +1956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>7</v>
       </c>
@@ -1797,7 +1975,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>7</v>
       </c>
@@ -1816,7 +1994,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
         <v>7</v>
       </c>
@@ -1835,7 +2013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="6" t="s">
         <v>7</v>
       </c>
@@ -1854,7 +2032,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="6" t="s">
         <v>7</v>
       </c>
@@ -1873,7 +2051,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="6" t="s">
         <v>7</v>
       </c>
@@ -1892,7 +2070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="6" t="s">
         <v>7</v>
       </c>
@@ -1911,7 +2089,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="6" t="s">
         <v>7</v>
       </c>
@@ -1932,6 +2110,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D64" xr:uid="{00000000-0009-0000-0000-000001000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="S02"/>
+      </filters>
+    </filterColumn>
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2520,7 +2703,9 @@
         <v>33</v>
       </c>
       <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
+      <c r="D10" s="8" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
@@ -2530,7 +2715,9 @@
         <v>34</v>
       </c>
       <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
+      <c r="D11" s="8" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
@@ -2539,7 +2726,9 @@
       <c r="B12" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="8"/>
+      <c r="C12" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="D12" s="8"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -2550,7 +2739,9 @@
         <v>36</v>
       </c>
       <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
+      <c r="D13" s="8" t="s">
+        <v>61</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:C13" xr:uid="{00000000-0009-0000-0000-000003000000}"/>

</xml_diff>

<commit_message>
data analysis metrics added to plot
</commit_message>
<xml_diff>
--- a/Data_Analysis/IMU_Results.xlsx
+++ b/Data_Analysis/IMU_Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALUMNO\Desktop\CEU\4\Proyectos\IMU_Visualization\Data_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB6A1CCB-E73D-4195-BBF4-51396C867B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF86A8DD-B956-47E6-AFB0-8E735EFA97E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subject_Metadata" sheetId="1" r:id="rId1"/>
@@ -388,7 +388,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -401,6 +401,9 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1236,7 +1239,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>6</v>
       </c>
@@ -1257,7 +1260,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>6</v>
       </c>
@@ -1279,7 +1282,7 @@
       </c>
       <c r="G24" s="10"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>6</v>
       </c>
@@ -1304,7 +1307,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>6</v>
       </c>
@@ -1325,7 +1328,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>6</v>
       </c>
@@ -1347,7 +1350,7 @@
       </c>
       <c r="G27" s="9"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>6</v>
       </c>
@@ -1369,7 +1372,7 @@
       </c>
       <c r="G28" s="9"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>6</v>
       </c>
@@ -1394,7 +1397,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>6</v>
       </c>
@@ -1422,7 +1425,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
         <v>6</v>
       </c>
@@ -1447,7 +1450,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
         <v>6</v>
       </c>
@@ -1468,7 +1471,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
         <v>6</v>
       </c>
@@ -1490,7 +1493,7 @@
       </c>
       <c r="G33" s="11"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
         <v>6</v>
       </c>
@@ -1512,7 +1515,7 @@
       </c>
       <c r="G34" s="11"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5" t="s">
         <v>6</v>
       </c>
@@ -1533,7 +1536,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
         <v>6</v>
       </c>
@@ -1558,7 +1561,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
         <v>6</v>
       </c>
@@ -1583,7 +1586,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
         <v>6</v>
       </c>
@@ -1602,7 +1605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
         <v>6</v>
       </c>
@@ -1627,7 +1630,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6" t="s">
         <v>6</v>
       </c>
@@ -1652,7 +1655,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
         <v>6</v>
       </c>
@@ -1671,7 +1674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6" t="s">
         <v>6</v>
       </c>
@@ -1690,7 +1693,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
         <v>6</v>
       </c>
@@ -1709,7 +1712,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
         <v>7</v>
       </c>
@@ -1728,7 +1731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="4" t="s">
         <v>7</v>
       </c>
@@ -1741,13 +1744,15 @@
       <c r="D45" s="4">
         <v>90</v>
       </c>
-      <c r="E45" s="4"/>
+      <c r="E45" s="4">
+        <v>82</v>
+      </c>
       <c r="F45" s="4">
         <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
         <v>7</v>
       </c>
@@ -1758,15 +1763,17 @@
         <v>16</v>
       </c>
       <c r="D46" s="4">
-        <v>180</v>
-      </c>
-      <c r="E46" s="4"/>
+        <v>145</v>
+      </c>
+      <c r="E46" s="4">
+        <v>137.30000000000001</v>
+      </c>
       <c r="F46" s="4">
         <f t="shared" si="0"/>
-        <v>180</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+        <v>7.6999999999999886</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
         <v>7</v>
       </c>
@@ -1779,13 +1786,15 @@
       <c r="D47" s="4">
         <v>0</v>
       </c>
-      <c r="E47" s="4"/>
+      <c r="E47" s="4">
+        <v>3.3</v>
+      </c>
       <c r="F47" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(D47-E47)</f>
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
         <v>7</v>
       </c>
@@ -1798,13 +1807,15 @@
       <c r="D48" s="4">
         <v>45</v>
       </c>
-      <c r="E48" s="4"/>
+      <c r="E48" s="4">
+        <v>55.2</v>
+      </c>
       <c r="F48" s="4">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E48-D48)</f>
+        <v>10.200000000000003</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="4" t="s">
         <v>7</v>
       </c>
@@ -1817,13 +1828,15 @@
       <c r="D49" s="4">
         <v>90</v>
       </c>
-      <c r="E49" s="4"/>
+      <c r="E49" s="4">
+        <v>86.4</v>
+      </c>
       <c r="F49" s="4">
-        <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E49-D49)</f>
+        <v>3.5999999999999943</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
         <v>7</v>
       </c>
@@ -1842,7 +1855,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
         <v>7</v>
       </c>
@@ -1861,7 +1874,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="s">
         <v>7</v>
       </c>
@@ -1880,7 +1893,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
         <v>7</v>
       </c>
@@ -1893,13 +1906,15 @@
       <c r="D53" s="5">
         <v>0</v>
       </c>
-      <c r="E53" s="5"/>
+      <c r="E53" s="5">
+        <v>5.4</v>
+      </c>
       <c r="F53" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
         <v>7</v>
       </c>
@@ -1912,13 +1927,15 @@
       <c r="D54" s="5">
         <v>90</v>
       </c>
-      <c r="E54" s="5"/>
+      <c r="E54" s="5">
+        <v>89.9</v>
+      </c>
       <c r="F54" s="5">
         <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>9.9999999999994316E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
         <v>7</v>
       </c>
@@ -1929,15 +1946,17 @@
         <v>16</v>
       </c>
       <c r="D55" s="5">
-        <v>145</v>
-      </c>
-      <c r="E55" s="5"/>
+        <v>143</v>
+      </c>
+      <c r="E55" s="5">
+        <v>134.30000000000001</v>
+      </c>
       <c r="F55" s="5">
         <f t="shared" si="0"/>
-        <v>145</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>8.6999999999999886</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
         <v>7</v>
       </c>
@@ -1950,13 +1969,13 @@
       <c r="D56" s="5">
         <v>0</v>
       </c>
-      <c r="E56" s="5"/>
+      <c r="E56" s="12"/>
       <c r="F56" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
         <v>7</v>
       </c>
@@ -1969,13 +1988,13 @@
       <c r="D57" s="5">
         <v>85</v>
       </c>
-      <c r="E57" s="5"/>
+      <c r="E57" s="12"/>
       <c r="F57" s="5">
         <f t="shared" si="0"/>
         <v>85</v>
       </c>
     </row>
-    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
         <v>7</v>
       </c>
@@ -1988,13 +2007,13 @@
       <c r="D58" s="5">
         <v>-85</v>
       </c>
-      <c r="E58" s="5"/>
+      <c r="E58" s="12"/>
       <c r="F58" s="5">
         <f t="shared" si="0"/>
         <v>85</v>
       </c>
     </row>
-    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
         <v>7</v>
       </c>
@@ -2007,13 +2026,13 @@
       <c r="D59" s="6">
         <v>0</v>
       </c>
-      <c r="E59" s="6"/>
+      <c r="E59" s="13"/>
       <c r="F59" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="6" t="s">
         <v>7</v>
       </c>
@@ -2026,13 +2045,13 @@
       <c r="D60" s="6">
         <v>70</v>
       </c>
-      <c r="E60" s="6"/>
+      <c r="E60" s="13"/>
       <c r="F60" s="6">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
     </row>
-    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="6" t="s">
         <v>7</v>
       </c>
@@ -2045,13 +2064,13 @@
       <c r="D61" s="6">
         <v>-70</v>
       </c>
-      <c r="E61" s="6"/>
+      <c r="E61" s="13"/>
       <c r="F61" s="6">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
     </row>
-    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="6" t="s">
         <v>7</v>
       </c>
@@ -2064,13 +2083,13 @@
       <c r="D62" s="6">
         <v>0</v>
       </c>
-      <c r="E62" s="6"/>
+      <c r="E62" s="13"/>
       <c r="F62" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="6" t="s">
         <v>7</v>
       </c>
@@ -2083,13 +2102,13 @@
       <c r="D63" s="6">
         <v>20</v>
       </c>
-      <c r="E63" s="6"/>
+      <c r="E63" s="13"/>
       <c r="F63" s="6">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="6" t="s">
         <v>7</v>
       </c>
@@ -2102,7 +2121,7 @@
       <c r="D64" s="6">
         <v>-30</v>
       </c>
-      <c r="E64" s="6"/>
+      <c r="E64" s="13"/>
       <c r="F64" s="6">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -2112,18 +2131,19 @@
   <autoFilter ref="A1:D64" xr:uid="{00000000-0009-0000-0000-000001000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="S02"/>
+        <filter val="S03"/>
       </filters>
     </filterColumn>
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr codeName="Hoja3"/>
+  <sheetPr codeName="Hoja3" filterMode="1"/>
   <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2156,7 +2176,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
@@ -2173,7 +2193,7 @@
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
@@ -2193,7 +2213,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
@@ -2213,7 +2233,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
@@ -2233,7 +2253,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
@@ -2250,7 +2270,7 @@
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
@@ -2267,7 +2287,7 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
@@ -2284,7 +2304,7 @@
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>5</v>
       </c>
@@ -2302,7 +2322,7 @@
       <c r="G9" s="5"/>
       <c r="I9" s="7"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>6</v>
       </c>
@@ -2319,7 +2339,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>6</v>
       </c>
@@ -2336,7 +2356,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>6</v>
       </c>
@@ -2353,7 +2373,7 @@
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>6</v>
       </c>
@@ -2370,7 +2390,7 @@
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>6</v>
       </c>
@@ -2387,7 +2407,7 @@
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>6</v>
       </c>
@@ -2404,7 +2424,7 @@
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>6</v>
       </c>
@@ -2421,7 +2441,7 @@
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>6</v>
       </c>
@@ -2536,9 +2556,15 @@
       <c r="D23" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
+      <c r="E23" s="5">
+        <v>17.12</v>
+      </c>
+      <c r="F23" s="5">
+        <v>34.39</v>
+      </c>
+      <c r="G23" s="5">
+        <v>0.98229999999999995</v>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
@@ -2555,7 +2581,7 @@
       </c>
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="G24" s="14"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
@@ -2575,8 +2601,15 @@
       <c r="G25" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D25" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:D25" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="S03"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Goniometer debug log change
</commit_message>
<xml_diff>
--- a/Data_Analysis/IMU_Results.xlsx
+++ b/Data_Analysis/IMU_Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALUMNO\Desktop\CEU\4\Proyectos\IMU_Visualization\Data_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6EDAC8-767E-4222-B3B3-C5A99D8BD810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C1D1357-0E74-4F79-A965-AD2DAA9CE6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subject_Metadata" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="63">
   <si>
     <t>Subject_ID</t>
   </si>
@@ -228,6 +228,9 @@
   </si>
   <si>
     <t>vamos a intentar hacerlo</t>
+  </si>
+  <si>
+    <t>Arturo Fierro</t>
   </si>
 </sst>
 </file>
@@ -750,8 +753,12 @@
       <c r="A5" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+      <c r="B5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>43</v>
+      </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>

</xml_diff>

<commit_message>
Data analysis changes and s04,s05,s06 calculations
</commit_message>
<xml_diff>
--- a/Data_Analysis/IMU_Results.xlsx
+++ b/Data_Analysis/IMU_Results.xlsx
@@ -8,20 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALUMNO\Desktop\CEU\4\Proyectos\IMU_Visualization\Data_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C1D1357-0E74-4F79-A965-AD2DAA9CE6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D86332D-DB55-410F-83A2-5A32F5154A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Subject_Metadata" sheetId="1" r:id="rId1"/>
     <sheet name="Static_Results" sheetId="2" r:id="rId2"/>
     <sheet name="Dynamic_Results" sheetId="3" r:id="rId3"/>
-    <sheet name="Complex_Results" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Complex_Results!$A$1:$C$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Dynamic_Results!$A$1:$D$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Static_Results!$A$1:$D$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Dynamic_Results!$A$1:$D$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Static_Results!$A$1:$D$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Subject_Metadata!$A$1:$C$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="52">
   <si>
     <t>Subject_ID</t>
   </si>
@@ -128,27 +126,6 @@
     <t>Fast</t>
   </si>
   <si>
-    <t>Activity</t>
-  </si>
-  <si>
-    <t>Pass/Fail</t>
-  </si>
-  <si>
-    <t>Observations</t>
-  </si>
-  <si>
-    <t>Touch Nose</t>
-  </si>
-  <si>
-    <t>Reach Doorknob</t>
-  </si>
-  <si>
-    <t>Pour Water</t>
-  </si>
-  <si>
-    <t>Comb Hair</t>
-  </si>
-  <si>
     <t>EXPECTED ERROR ENTRE 2º Y 5º</t>
   </si>
   <si>
@@ -176,24 +153,6 @@
     <t>Male</t>
   </si>
   <si>
-    <t>pass</t>
-  </si>
-  <si>
-    <t>muy preciso</t>
-  </si>
-  <si>
-    <t>with palm touches face, not fingers</t>
-  </si>
-  <si>
-    <t>desviacion a la izquierda, descordinacion radial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hiperflexion radiocubital </t>
-  </si>
-  <si>
-    <t>ligera desviacion radial izquierda</t>
-  </si>
-  <si>
     <t>Macarena Querol</t>
   </si>
   <si>
@@ -231,6 +190,12 @@
   </si>
   <si>
     <t>Arturo Fierro</t>
+  </si>
+  <si>
+    <t>Iñigo Gonzalez</t>
+  </si>
+  <si>
+    <t>Alvaro Sanchez</t>
   </si>
 </sst>
 </file>
@@ -268,7 +233,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -311,12 +276,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -345,7 +304,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -354,7 +313,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -674,7 +632,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -694,10 +652,10 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D2" s="2">
         <v>178</v>
@@ -714,10 +672,10 @@
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D3" s="3">
         <v>195</v>
@@ -734,10 +692,10 @@
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D4" s="2">
         <v>176</v>
@@ -751,13 +709,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -765,27 +723,35 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
+        <v>39</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
+        <v>40</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -795,7 +761,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -805,7 +771,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -825,7 +791,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Hoja2" filterMode="1"/>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="16.7265625" customWidth="1"/>
@@ -892,7 +858,7 @@
         <v>90</v>
       </c>
       <c r="H3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
@@ -1427,7 +1393,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>7</v>
       </c>
@@ -1448,7 +1414,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>7</v>
       </c>
@@ -1469,7 +1435,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
         <v>7</v>
       </c>
@@ -1490,7 +1456,7 @@
         <v>7.6999999999999886</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
         <v>7</v>
       </c>
@@ -1511,7 +1477,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
         <v>7</v>
       </c>
@@ -1532,7 +1498,7 @@
         <v>10.200000000000003</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
         <v>7</v>
       </c>
@@ -1553,7 +1519,7 @@
         <v>3.5999999999999943</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
         <v>7</v>
       </c>
@@ -1574,7 +1540,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
         <v>7</v>
       </c>
@@ -1595,7 +1561,7 @@
         <v>9.9999999999994316E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
         <v>7</v>
       </c>
@@ -1616,7 +1582,7 @@
         <v>8.6999999999999886</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
         <v>7</v>
       </c>
@@ -1635,10 +1601,10 @@
         <v>0</v>
       </c>
       <c r="H41" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
         <v>7</v>
       </c>
@@ -1657,7 +1623,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5" t="s">
         <v>7</v>
       </c>
@@ -1676,7 +1642,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6" t="s">
         <v>7</v>
       </c>
@@ -1695,7 +1661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6" t="s">
         <v>7</v>
       </c>
@@ -1714,10 +1680,10 @@
         <v>70</v>
       </c>
       <c r="H45" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="6" t="s">
         <v>7</v>
       </c>
@@ -1736,9 +1702,9 @@
         <v>70</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>13</v>
@@ -1749,15 +1715,14 @@
       <c r="D47" s="4">
         <v>0</v>
       </c>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E47" s="4">
+        <v>0.9</v>
+      </c>
+      <c r="F47" s="4"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>13</v>
@@ -1768,15 +1733,17 @@
       <c r="D48" s="4">
         <v>90</v>
       </c>
-      <c r="E48" s="4"/>
+      <c r="E48" s="4">
+        <v>75.900000000000006</v>
+      </c>
       <c r="F48" s="4">
         <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>14.099999999999994</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>13</v>
@@ -1785,17 +1752,19 @@
         <v>16</v>
       </c>
       <c r="D49" s="4">
-        <v>180</v>
-      </c>
-      <c r="E49" s="4"/>
+        <v>150</v>
+      </c>
+      <c r="E49" s="4">
+        <v>150.4</v>
+      </c>
       <c r="F49" s="4">
         <f t="shared" ref="F49:F76" si="1">ABS(E49-D49)</f>
-        <v>180</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>0.40000000000000568</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>13</v>
@@ -1806,15 +1775,17 @@
       <c r="D50" s="4">
         <v>0</v>
       </c>
-      <c r="E50" s="4"/>
+      <c r="E50" s="4">
+        <v>0.5</v>
+      </c>
       <c r="F50" s="4">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>13</v>
@@ -1825,15 +1796,17 @@
       <c r="D51" s="4">
         <v>45</v>
       </c>
-      <c r="E51" s="4"/>
+      <c r="E51" s="4">
+        <v>44.4</v>
+      </c>
       <c r="F51" s="4">
-        <f t="shared" si="1"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E51-E50-D51)</f>
+        <v>1.1000000000000014</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>13</v>
@@ -1844,15 +1817,17 @@
       <c r="D52" s="4">
         <v>90</v>
       </c>
-      <c r="E52" s="4"/>
+      <c r="E52" s="4">
+        <v>74.099999999999994</v>
+      </c>
       <c r="F52" s="4">
-        <f t="shared" si="1"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E52-E50-D52)</f>
+        <v>16.400000000000006</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>14</v>
@@ -1863,15 +1838,14 @@
       <c r="D53" s="5">
         <v>0</v>
       </c>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E53" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="F53" s="5"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>14</v>
@@ -1882,15 +1856,17 @@
       <c r="D54" s="5">
         <v>90</v>
       </c>
-      <c r="E54" s="5"/>
+      <c r="E54" s="5">
+        <v>72.900000000000006</v>
+      </c>
       <c r="F54" s="5">
-        <f t="shared" si="1"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E54-E53-D54)</f>
+        <v>17.599999999999994</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>14</v>
@@ -1899,17 +1875,19 @@
         <v>16</v>
       </c>
       <c r="D55" s="5">
-        <v>145</v>
-      </c>
-      <c r="E55" s="5"/>
+        <v>133</v>
+      </c>
+      <c r="E55" s="5">
+        <v>122.6</v>
+      </c>
       <c r="F55" s="5">
-        <f t="shared" si="1"/>
-        <v>145</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E55-E53-D55)</f>
+        <v>10.900000000000006</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>14</v>
@@ -1920,15 +1898,14 @@
       <c r="D56" s="5">
         <v>0</v>
       </c>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E56" s="5">
+        <v>35.799999999999997</v>
+      </c>
+      <c r="F56" s="5"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>14</v>
@@ -1939,15 +1916,17 @@
       <c r="D57" s="5">
         <v>85</v>
       </c>
-      <c r="E57" s="5"/>
+      <c r="E57" s="5">
+        <v>96</v>
+      </c>
       <c r="F57" s="5">
-        <f t="shared" si="1"/>
-        <v>85</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(D57-(E57-E56))</f>
+        <v>24.799999999999997</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>14</v>
@@ -1956,17 +1935,19 @@
         <v>18</v>
       </c>
       <c r="D58" s="5">
-        <v>85</v>
-      </c>
-      <c r="E58" s="5"/>
+        <v>-85</v>
+      </c>
+      <c r="E58" s="5">
+        <v>-53</v>
+      </c>
       <c r="F58" s="5">
-        <f t="shared" si="1"/>
-        <v>85</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(D58-(E58-E56))</f>
+        <v>3.7999999999999972</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B59" s="6" t="s">
         <v>15</v>
@@ -1977,15 +1958,14 @@
       <c r="D59" s="6">
         <v>0</v>
       </c>
-      <c r="E59" s="6"/>
-      <c r="F59" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E59" s="6">
+        <v>-9.9</v>
+      </c>
+      <c r="F59" s="6"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="6" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>15</v>
@@ -1996,15 +1976,17 @@
       <c r="D60" s="6">
         <v>70</v>
       </c>
-      <c r="E60" s="6"/>
+      <c r="E60" s="6">
+        <v>60.7</v>
+      </c>
       <c r="F60" s="6">
-        <f t="shared" si="1"/>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E60-E59-D60)</f>
+        <v>0.60000000000000853</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="6" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B61" s="6" t="s">
         <v>15</v>
@@ -2015,15 +1997,17 @@
       <c r="D61" s="6">
         <v>-70</v>
       </c>
-      <c r="E61" s="6"/>
+      <c r="E61" s="6">
+        <v>-68.5</v>
+      </c>
       <c r="F61" s="6">
-        <f t="shared" si="1"/>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E61-E59-D61)</f>
+        <v>11.399999999999999</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B62" s="4" t="s">
         <v>13</v>
@@ -2034,15 +2018,14 @@
       <c r="D62" s="4">
         <v>0</v>
       </c>
-      <c r="E62" s="4"/>
-      <c r="F62" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E62" s="4">
+        <v>0.3</v>
+      </c>
+      <c r="F62" s="4"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>13</v>
@@ -2053,15 +2036,17 @@
       <c r="D63" s="4">
         <v>90</v>
       </c>
-      <c r="E63" s="4"/>
+      <c r="E63" s="4">
+        <v>80.5</v>
+      </c>
       <c r="F63" s="4">
-        <f t="shared" si="1"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E63-E62-D63)</f>
+        <v>9.7999999999999972</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>13</v>
@@ -2070,17 +2055,19 @@
         <v>16</v>
       </c>
       <c r="D64" s="4">
-        <v>180</v>
-      </c>
-      <c r="E64" s="4"/>
+        <v>140</v>
+      </c>
+      <c r="E64" s="4">
+        <v>129.30000000000001</v>
+      </c>
       <c r="F64" s="4">
-        <f t="shared" si="1"/>
-        <v>180</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E64-E62-D64)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>13</v>
@@ -2091,15 +2078,14 @@
       <c r="D65" s="4">
         <v>0</v>
       </c>
-      <c r="E65" s="4"/>
-      <c r="F65" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E65" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="F65" s="4"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>13</v>
@@ -2110,15 +2096,17 @@
       <c r="D66" s="4">
         <v>45</v>
       </c>
-      <c r="E66" s="4"/>
+      <c r="E66" s="4">
+        <v>50.8</v>
+      </c>
       <c r="F66" s="4">
-        <f t="shared" si="1"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E66-E65-D66)</f>
+        <v>4.2999999999999972</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>13</v>
@@ -2129,15 +2117,17 @@
       <c r="D67" s="4">
         <v>90</v>
       </c>
-      <c r="E67" s="4"/>
+      <c r="E67" s="4">
+        <v>79.900000000000006</v>
+      </c>
       <c r="F67" s="4">
-        <f t="shared" si="1"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E67-E65-D67)</f>
+        <v>11.599999999999994</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>14</v>
@@ -2148,15 +2138,14 @@
       <c r="D68" s="5">
         <v>0</v>
       </c>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E68" s="5">
+        <v>1.3</v>
+      </c>
+      <c r="F68" s="5"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>14</v>
@@ -2167,15 +2156,17 @@
       <c r="D69" s="5">
         <v>90</v>
       </c>
-      <c r="E69" s="5"/>
+      <c r="E69" s="5">
+        <v>76.7</v>
+      </c>
       <c r="F69" s="5">
-        <f t="shared" si="1"/>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E69-E68-D69)</f>
+        <v>14.599999999999994</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>14</v>
@@ -2186,15 +2177,17 @@
       <c r="D70" s="5">
         <v>145</v>
       </c>
-      <c r="E70" s="5"/>
+      <c r="E70" s="5">
+        <v>104.9</v>
+      </c>
       <c r="F70" s="5">
-        <f t="shared" si="1"/>
-        <v>145</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E70-E68-D70)</f>
+        <v>41.399999999999991</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>14</v>
@@ -2205,15 +2198,17 @@
       <c r="D71" s="5">
         <v>0</v>
       </c>
-      <c r="E71" s="5"/>
+      <c r="E71" s="5">
+        <v>7.9</v>
+      </c>
       <c r="F71" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>14</v>
@@ -2224,15 +2219,17 @@
       <c r="D72" s="5">
         <v>85</v>
       </c>
-      <c r="E72" s="5"/>
+      <c r="E72" s="5">
+        <v>89.7</v>
+      </c>
       <c r="F72" s="5">
-        <f t="shared" si="1"/>
-        <v>85</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E72-E71-D72)</f>
+        <v>3.2000000000000028</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>14</v>
@@ -2241,17 +2238,19 @@
         <v>18</v>
       </c>
       <c r="D73" s="5">
-        <v>85</v>
-      </c>
-      <c r="E73" s="5"/>
+        <v>-85</v>
+      </c>
+      <c r="E73" s="5">
+        <v>-64.400000000000006</v>
+      </c>
       <c r="F73" s="5">
-        <f t="shared" si="1"/>
-        <v>85</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E73-E71-D73)</f>
+        <v>12.699999999999989</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="6" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B74" s="6" t="s">
         <v>15</v>
@@ -2262,15 +2261,14 @@
       <c r="D74" s="6">
         <v>0</v>
       </c>
-      <c r="E74" s="6"/>
-      <c r="F74" s="6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+      <c r="E74" s="6">
+        <v>-4.7</v>
+      </c>
+      <c r="F74" s="6"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="6" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B75" s="6" t="s">
         <v>15</v>
@@ -2281,15 +2279,17 @@
       <c r="D75" s="6">
         <v>70</v>
       </c>
-      <c r="E75" s="6"/>
+      <c r="E75" s="6">
+        <v>56.9</v>
+      </c>
       <c r="F75" s="6">
-        <f t="shared" si="1"/>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <f>ABS(E75-E74-D75)</f>
+        <v>8.3999999999999986</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="6" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B76" s="6" t="s">
         <v>15</v>
@@ -2300,17 +2300,321 @@
       <c r="D76" s="6">
         <v>-70</v>
       </c>
-      <c r="E76" s="6"/>
+      <c r="E76" s="6">
+        <v>-74.900000000000006</v>
+      </c>
       <c r="F76" s="6">
-        <f t="shared" si="1"/>
+        <f>ABS(E76-E74-D76)</f>
+        <v>0.20000000000000284</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A77" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D77" s="4">
+        <v>0</v>
+      </c>
+      <c r="E77" s="4">
+        <v>0.2</v>
+      </c>
+      <c r="F77" s="4"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A78" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D78" s="4">
+        <v>90</v>
+      </c>
+      <c r="E78" s="4">
+        <v>88.8</v>
+      </c>
+      <c r="F78" s="4">
+        <f>ABS(E78-E77-D78)</f>
+        <v>1.4000000000000057</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D79" s="4">
+        <v>150</v>
+      </c>
+      <c r="E79" s="4">
+        <v>167.1</v>
+      </c>
+      <c r="F79" s="4">
+        <f>ABS(E79-E77-D79)</f>
+        <v>16.900000000000006</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A80" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D80" s="4">
+        <v>0</v>
+      </c>
+      <c r="E80" s="4">
+        <v>0.2</v>
+      </c>
+      <c r="F80" s="4"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A81" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D81" s="4">
+        <v>45</v>
+      </c>
+      <c r="E81" s="4">
+        <v>40.6</v>
+      </c>
+      <c r="F81" s="4">
+        <f>ABS(E81-E80-D81)</f>
+        <v>4.6000000000000014</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A82" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D82" s="4">
+        <v>90</v>
+      </c>
+      <c r="E82" s="4">
+        <v>79.3</v>
+      </c>
+      <c r="F82" s="4">
+        <f>ABS(E82-E80-D82)</f>
+        <v>10.900000000000006</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A83" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B83" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C83" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D83" s="5">
+        <v>0</v>
+      </c>
+      <c r="E83" s="5">
+        <v>1.8</v>
+      </c>
+      <c r="F83" s="5"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A84" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B84" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D84" s="5">
+        <v>90</v>
+      </c>
+      <c r="E84" s="5">
+        <v>81.400000000000006</v>
+      </c>
+      <c r="F84" s="5">
+        <f>ABS(E84-E83-D84)</f>
+        <v>10.399999999999991</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A85" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C85" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D85" s="5">
+        <v>135</v>
+      </c>
+      <c r="E85" s="5">
+        <v>126.6</v>
+      </c>
+      <c r="F85" s="5">
+        <f>ABS(E85-E83-D85)</f>
+        <v>10.200000000000003</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A86" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B86" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D86" s="5">
+        <v>0</v>
+      </c>
+      <c r="E86" s="5">
+        <v>15.9</v>
+      </c>
+      <c r="F86" s="5"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A87" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D87" s="5">
+        <v>85</v>
+      </c>
+      <c r="E87" s="5">
+        <v>83.9</v>
+      </c>
+      <c r="F87" s="5">
+        <f>ABS(E87-E86-D87)</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A88" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D88" s="5">
+        <v>-85</v>
+      </c>
+      <c r="E88" s="5">
+        <v>-71.099999999999994</v>
+      </c>
+      <c r="F88" s="5">
+        <f>ABS(E88-E86-D88)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D89" s="6">
+        <v>0</v>
+      </c>
+      <c r="E89" s="6">
+        <v>-16.7</v>
+      </c>
+      <c r="F89" s="6"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D90" s="6">
         <v>70</v>
       </c>
+      <c r="E90" s="6">
+        <v>45.9</v>
+      </c>
+      <c r="F90" s="6">
+        <f>ABS(E90-E89-D90)</f>
+        <v>7.4000000000000057</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B91" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D91" s="6">
+        <v>-50</v>
+      </c>
+      <c r="E91" s="6">
+        <v>-47.1</v>
+      </c>
+      <c r="F91" s="6">
+        <f>ABS(E91-E89-D91)</f>
+        <v>19.599999999999998</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D76" xr:uid="{00000000-0009-0000-0000-000001000000}">
+  <autoFilter ref="A1:D91" xr:uid="{00000000-0009-0000-0000-000001000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="S03"/>
+        <filter val="S04"/>
+        <filter val="S05"/>
+        <filter val="S06"/>
       </filters>
     </filterColumn>
     <filterColumn colId="3" hiddenButton="1"/>
@@ -2323,8 +2627,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr codeName="Hoja3"/>
-  <dimension ref="A1:L41"/>
+  <sheetPr codeName="Hoja3" filterMode="1"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="16.7265625" customWidth="1"/>
@@ -2356,7 +2660,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
@@ -2373,10 +2677,10 @@
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="I2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
@@ -2393,10 +2697,10 @@
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="L3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
@@ -2413,13 +2717,13 @@
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="I4" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="L4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
@@ -2436,10 +2740,10 @@
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="L5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
@@ -2456,7 +2760,7 @@
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
@@ -2473,7 +2777,7 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>5</v>
       </c>
@@ -2490,10 +2794,10 @@
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
       <c r="I8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>5</v>
       </c>
@@ -2511,7 +2815,7 @@
       <c r="G9" s="5"/>
       <c r="I9" s="7"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>6</v>
       </c>
@@ -2528,7 +2832,7 @@
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>6</v>
       </c>
@@ -2545,7 +2849,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>6</v>
       </c>
@@ -2562,7 +2866,7 @@
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>6</v>
       </c>
@@ -2579,7 +2883,7 @@
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>6</v>
       </c>
@@ -2596,7 +2900,7 @@
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
         <v>6</v>
       </c>
@@ -2613,7 +2917,7 @@
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
         <v>6</v>
       </c>
@@ -2630,7 +2934,7 @@
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>6</v>
       </c>
@@ -2647,7 +2951,7 @@
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>7</v>
       </c>
@@ -2664,7 +2968,7 @@
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>7</v>
       </c>
@@ -2681,7 +2985,7 @@
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>7</v>
       </c>
@@ -2698,7 +3002,7 @@
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>7</v>
       </c>
@@ -2715,7 +3019,7 @@
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
         <v>7</v>
       </c>
@@ -2738,7 +3042,7 @@
         <v>0.98270000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5" t="s">
         <v>7</v>
       </c>
@@ -2761,7 +3065,7 @@
         <v>0.97789999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>7</v>
       </c>
@@ -2776,12 +3080,12 @@
       </c>
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
-      <c r="G24" s="9"/>
+      <c r="G24" s="8"/>
       <c r="I24" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>7</v>
       </c>
@@ -2800,7 +3104,7 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>13</v>
@@ -2817,7 +3121,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>13</v>
@@ -2834,7 +3138,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>13</v>
@@ -2851,7 +3155,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>13</v>
@@ -2868,7 +3172,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>14</v>
@@ -2885,7 +3189,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>14</v>
@@ -2902,7 +3206,7 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>14</v>
@@ -2915,11 +3219,11 @@
       </c>
       <c r="E32" s="5"/>
       <c r="F32" s="5"/>
-      <c r="G32" s="9"/>
+      <c r="G32" s="8"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="5" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>14</v>
@@ -2936,7 +3240,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>13</v>
@@ -2953,7 +3257,7 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>13</v>
@@ -2970,7 +3274,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>13</v>
@@ -2987,7 +3291,7 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>13</v>
@@ -3004,7 +3308,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>14</v>
@@ -3021,7 +3325,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>14</v>
@@ -3038,7 +3342,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>14</v>
@@ -3051,11 +3355,11 @@
       </c>
       <c r="E40" s="5"/>
       <c r="F40" s="5"/>
-      <c r="G40" s="9"/>
+      <c r="G40" s="8"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="5" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>14</v>
@@ -3070,179 +3374,153 @@
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
     </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="4"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A46" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A47" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A48" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="8"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A49" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D25" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:D41" xr:uid="{00000000-0009-0000-0000-000002000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="S04"/>
+        <filter val="S05"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <sheetPr codeName="Hoja4"/>
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="4" width="16.7265625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="3"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="8"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:C13" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>